<commit_message>
THE glucuronide isomers I/II in Table 2 (full and compact), Table S3 and Fig. 3 panel titles
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WDn5T1yz4TRFaKpaKqad5Y
</commit_message>
<xml_diff>
--- a/submission_analytica/2_main_tables/Table2_compact.xlsx
+++ b/submission_analytica/2_main_tables/Table2_compact.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="42">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="43">
   <si>
     <t>No.</t>
   </si>
@@ -44,7 +44,10 @@
     <t>11-Oxoetiocholanolone glucuronide* (3)</t>
   </si>
   <si>
-    <t>Tetrahydrocortisone glucuronide† (3)</t>
+    <t>Tetrahydrocortisone glucuronide, isomer I† (3)</t>
+  </si>
+  <si>
+    <t>Tetrahydrocortisone glucuronide, isomer II† (3)</t>
   </si>
   <si>
     <t>Biliverdin (2)</t>
@@ -140,7 +143,7 @@
     <t>Table 2. Annotated bladder-cancer findings (BC vs Control; MSI levels 2–3). log2FC and q (Benjamini–Hochberg), linear model adjusted for sex, age and the exogenous-signal index; AUC, all samples; p (matched), Mann–Whitney U test in age- and sex-matched subsets. Finding criteria are given in Section 2.5; complete statistics are in Table S1 and annotation details in Table S3.</t>
   </si>
   <si>
-    <t>* 5α-Isomer (11-oxoandrosterone glucuronide) not excluded; identity assigned from the aglycone MS/MS. † Two chromatographically resolved isomers; allo-tetrahydrocortisone and 3- vs 21-glucuronide not excluded. Isomers not excluded for the other compounds are listed in Table S3.</t>
+    <t>* 5α-Isomer (11-oxoandrosterone glucuronide) not excluded; identity assigned from the aglycone MS/MS. † Isomers I and II are chromatographically resolved (11.06 and 10.76 min); allo-tetrahydrocortisone and 3- vs 21-glucuronide not excluded. Isomers not excluded for the other compounds are listed in Table S3.</t>
   </si>
 </sst>
 </file>
@@ -509,22 +512,22 @@
         <v>8</v>
       </c>
       <c r="C2" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="D2" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E2" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="F2" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="G2" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="H2" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
     </row>
     <row r="3" spans="1:8">
@@ -535,22 +538,22 @@
         <v>9</v>
       </c>
       <c r="C3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="D3" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="E3" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="F3" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="G3" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="H3" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
     </row>
     <row r="4" spans="1:8">
@@ -558,25 +561,25 @@
         <v>3</v>
       </c>
       <c r="B4" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="C4" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="D4" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="E4" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="F4" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="G4" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="H4" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
     </row>
     <row r="5" spans="1:8">
@@ -584,25 +587,25 @@
         <v>4</v>
       </c>
       <c r="B5" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="C5" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="D5" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="E5" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="F5" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="G5" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="H5" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
     </row>
     <row r="6" spans="1:8">
@@ -610,25 +613,25 @@
         <v>5</v>
       </c>
       <c r="B6" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="C6" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="D6" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="E6" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="F6" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="G6" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="H6" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
     </row>
   </sheetData>
@@ -643,12 +646,12 @@
   <sheetData>
     <row r="1" spans="1:1">
       <c r="A1" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
     </row>
     <row r="2" spans="1:1">
       <c r="A2" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
     </row>
   </sheetData>

</xml_diff>